<commit_message>
Update Session Plan: 10 sessions x 3hrs, TEJAS JADHAV CFA FRM MMS(SIMSREE), no Jupyter Notebook
- Restructured from 20x1.5hr to 10 sessions x 3 hours (Hour 1 / Hour 2 / Hour 3-Lab per module)
- Faculty name updated to: TEJAS JADHAV, CFA, FRM | MMS (SIMSREE) Mumbai
- Removed all Jupyter Notebook references; replaced with Python (VS Code) and Python script
- Excel and PDF regenerated to match

https://claude.ai/code/session_01MUJzDraqNW46ThEJmDubED
</commit_message>
<xml_diff>
--- a/Session_Plan_PGDM_2025-27_Sem3_AI_Finance.xlsx
+++ b/Session_Plan_PGDM_2025-27_Sem3_AI_Finance.xlsx
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B7" s="92" t="inlineStr">
         <is>
-          <t>Tejas Jadhav | CFA Charterholder, FRM Certified</t>
+          <t>TEJAS JADHAV, CFA, FRM | MMS (SIMSREE) Mumbai</t>
         </is>
       </c>
       <c r="C7" s="93" t="n"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B8" s="92" t="inlineStr">
         <is>
-          <t>"Agentic AI &amp; Advanced Analytics in Finance" is a 30-hour Semester III PGDM specialization designed to equip students with production-grade AI and quantitative skills sought by Global Capability Centres (GCCs) and financial institutions. The course covers agentic AI architectures, prompt engineering, RAG pipelines, algorithmic trading, Monte Carlo VaR, Basel III/IV compliance automation, and fund administration workflows. Drawing from Harvard Case Method, NUS sandbox-first pedagogy, GARP FRM frameworks, and CFA Institute standards, each module delivers a deployable project artifact that builds the student's live portfolio. The capstone simulates a real GCC hiring panel, ensuring placement readiness upon completion.</t>
+          <t>"Agentic AI &amp; Advanced Analytics in Finance" is a 30-hour PGDM Semester III specialization equipping students with production-grade AI and quantitative finance skills sought by Global Capability Centres and financial institutions. The course covers agentic AI architectures, prompt engineering, RAG pipelines, algorithmic trading, Monte Carlo VaR, Basel III/IV compliance automation, and fund administration workflows. Drawing from Harvard Case Method, NUS sandbox-first pedagogy, GARP FRM frameworks, and CFA Institute standards, each of the 10 modules (3 hours each) delivers a deployable project artifact building the student's live portfolio. The capstone simulates a real GCC hiring panel, ensuring placement readiness upon completion.</t>
         </is>
       </c>
       <c r="C8" s="93" t="n"/>
@@ -1526,7 +1526,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Module 1: Foundations of Agentic AI in Financial Services</t>
+          <t>Session 1 (3 hrs) | Module 1: Foundations of Agentic AI in Financial Services</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C20" s="79" t="inlineStr">
         <is>
-          <t>LLM Fundamentals &amp; Financial AI Overview: Introduction to Large Language Models; transformer architecture and attention mechanism; tokenization and embeddings; evolution from rule-based to neural to agentic AI in financial services; Bloomberg GPT, FinBERT, and Claude API applications in finance.</t>
+          <t>[Hour 1] LLM Fundamentals &amp; Financial AI Overview: Transformer architecture, attention mechanism, tokenization; evolution of AI in finance (rule-based → ML → agentic); Bloomberg GPT, FinBERT, Claude API applications in financial services.</t>
         </is>
       </c>
       <c r="D20" s="80" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="C21" s="83" t="inlineStr">
         <is>
-          <t>Financial NLP Applications &amp; Data APIs: Named Entity Recognition (NER) for financial data; text classification of annual reports and regulatory filings; SEBI filing structure; financial data APIs (NSE, BSE, Yahoo Finance, RBI DBIE); structured vs. unstructured financial data challenges.</t>
+          <t>[Hour 2] Agentic AI Architecture: Observe-Plan-Act-Reflect agent loop; tool definitions and function calling; agent memory types (short-term, episodic, semantic, procedural); financial data APIs — NSE, BSE, Yahoo Finance, RBI DBIE.</t>
         </is>
       </c>
       <c r="D21" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Live Demo (Yahoo Finance API); Case Excerpt: 'Morgan Stanley GPT-4 Wealth Advisor Program'</t>
+          <t>Lecture + Live Demo; Case: 'Morgan Stanley GPT-4 Wealth Advisor Program'</t>
         </is>
       </c>
     </row>
@@ -1566,19 +1566,19 @@
       </c>
       <c r="C22" s="83" t="inlineStr">
         <is>
-          <t>Agentic AI Architecture &amp; Lab: Observe-Plan-Act-Reflect agent loop; tool definitions and function calling; agent memory types (short-term, episodic, semantic, procedural); Lab: Build a structured financial data extraction prompt using the Claude API to extract income statement data from unstructured text.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a structured financial data extraction prompt using Claude API and Python (VS Code) — extract income statement line items from 3 different annual report excerpts; compare output quality across prompt patterns.</t>
         </is>
       </c>
       <c r="D22" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (Python + Anthropic Claude API); Instructor Demo; Peer Discussion</t>
+          <t>In-Class Python Lab (VS Code + Claude API); Instructor Demo; Peer Discussion</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>Module 2: Prompt Engineering &amp; RAG for Financial Analysis</t>
+          <t>Session 2 (3 hrs) | Module 2: Prompt Engineering &amp; RAG for Financial Analysis</t>
         </is>
       </c>
       <c r="B23" s="21" t="n">
@@ -1586,12 +1586,12 @@
       </c>
       <c r="C23" s="83" t="inlineStr">
         <is>
-          <t>Prompt Engineering Fundamentals: Zero-shot, one-shot, few-shot prompting patterns; chain-of-thought (CoT) prompting for financial reasoning; role prompting ('You are a CFO analyzing...'); system prompt architecture; output formatting (JSON, markdown tables); prompt templating best practices.</t>
+          <t>[Hour 1] Prompt Engineering for Finance: Zero-shot, few-shot, chain-of-thought (CoT) prompting; role prompting; output formatting (JSON, markdown tables); hallucination risks; Group Activity: redesign five failing financial prompts.</t>
         </is>
       </c>
       <c r="D23" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Live Prompting Exercise; Pair Activity: compare prompt outputs for same financial query</t>
+          <t>Lecture + Live Prompting Exercise; Pair Activity: compare prompt outputs; Group Redesign Workshop</t>
         </is>
       </c>
     </row>
@@ -1602,12 +1602,12 @@
       </c>
       <c r="C24" s="24" t="inlineStr">
         <is>
-          <t>Advanced Prompting &amp; Failure Mode Analysis: Self-consistency and tree-of-thought prompting; hallucination risks in financial AI outputs and mitigation strategies; prompt injection awareness; common failure patterns in financial prompts; Group Activity: redesign five failing financial prompts.</t>
+          <t>[Hour 2] RAG Pipeline Construction: Vector databases (ChromaDB, Pinecone); document chunking for financial docs; embedding models (Sentence Transformers); retrieval and re-ranking; advanced prompting — self-consistency, tree-of-thought.</t>
         </is>
       </c>
       <c r="D24" s="25" t="inlineStr">
         <is>
-          <t>Group Workshop (Prompt Redesign); Peer Review; Class Discussion on AI reliability in finance</t>
+          <t>Lecture; Architecture Diagram Workshop; Industry Application: 'SEBI DRHP Analysis using RAG'</t>
         </is>
       </c>
     </row>
@@ -1618,19 +1618,19 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>RAG Pipeline Construction Lab: Vector database concepts (ChromaDB, Pinecone, Weaviate); document chunking strategies for financial documents; embedding models (Sentence Transformers); retrieval and re-ranking; Lab: Build a Q&amp;A bot on a 200-page NSE IPO Prospectus using LlamaIndex and Claude API.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a Q&amp;A bot on a 200-page NSE IPO Prospectus using LlamaIndex + ChromaDB + Claude API (VS Code); test with 10 investor questions; evaluate retrieval accuracy; peer review output.</t>
         </is>
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
-          <t>Sandbox Lab (LlamaIndex + ChromaDB + Claude API); Industry Application: 'SEBI DRHP Analysis using RAG'</t>
+          <t>In-Class Python Lab (VS Code + LlamaIndex + ChromaDB + Claude API); Peer Review</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>Module 3: Model Context Protocol &amp; Agent Orchestration</t>
+          <t>Session 3 (3 hrs) | Module 3: Model Context Protocol &amp; Agent Orchestration</t>
         </is>
       </c>
       <c r="B26" s="17" t="n">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C26" s="79" t="inlineStr">
         <is>
-          <t>Model Context Protocol (MCP) Architecture: MCP protocol specification; tool definitions and JSON schemas; context window management for long financial documents; memory management (summarization, rolling context); financial context design patterns: credit analyst agent, portfolio manager agent.</t>
+          <t>[Hour 1] Model Context Protocol (MCP): Protocol specification; tool definitions and JSON schemas; context window management for long financial documents; memory management (summarization, rolling context); financial context design patterns.</t>
         </is>
       </c>
       <c r="D26" s="80" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C27" s="83" t="inlineStr">
         <is>
-          <t>Multi-Agent Frameworks – CrewAI &amp; LangGraph: Introduction to CrewAI and LangGraph; agent roles (researcher, analyst, writer, reviewer); sequential vs. hierarchical vs. parallel workflows; inter-agent communication protocols; designing agent crews for financial tasks (due diligence, investment research).</t>
+          <t>[Hour 2] Multi-Agent Frameworks: CrewAI and LangGraph; agent roles (researcher, analyst, writer, reviewer); sequential vs. hierarchical vs. parallel workflows; inter-agent communication; designing agent crews for financial due diligence.</t>
         </is>
       </c>
       <c r="D27" s="84" t="inlineStr">
@@ -1670,19 +1670,19 @@
       </c>
       <c r="C28" s="83" t="inlineStr">
         <is>
-          <t>Multi-Agent Investment Memo Lab: Lab – Build a 3-agent Investment Memo pipeline: Research Agent (data gathering and summarization) → Analysis Agent (financial modelling and interpretation) → Writing Agent (memo drafting); agent evaluation metrics; quality assurance frameworks; deployment considerations.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a 3-agent Investment Memo pipeline — Research Agent (data gathering) → Analysis Agent (interpretation) → Writing Agent (memo drafting); run on a real NSE-listed company; peer review memo quality against IB standards.</t>
         </is>
       </c>
       <c r="D28" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (CrewAI + Claude API); Peer Review Panel (evaluate memo quality against investment banking standards)</t>
+          <t>In-Class Python Lab (VS Code + CrewAI + Claude API); Peer Review Panel</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Module 4: Algorithmic Trading &amp; Execution Strategies</t>
+          <t>Session 4 (3 hrs) | Module 4: Algorithmic Trading &amp; Execution Strategies</t>
         </is>
       </c>
       <c r="B29" s="21" t="n">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="C29" s="83" t="inlineStr">
         <is>
-          <t>Market Microstructure &amp; Trading Signals: Order book dynamics, bid-ask spread, market depth; order types (market, limit, stop-loss, IOC); trading signal categories – momentum (RSI, MACD), mean-reversion (Bollinger Bands), statistical arbitrage (pairs trading, cointegration); SEBI algorithmic trading and co-location guidelines.</t>
+          <t>[Hour 1] Market Microstructure &amp; Trading Signals: Order book dynamics, bid-ask spread, order types; momentum (RSI, MACD), mean-reversion (Bollinger Bands), pairs trading (cointegration); SEBI algorithmic trading and co-location guidelines.</t>
         </is>
       </c>
       <c r="D29" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Simulation Exercise (virtual order book); Case Excerpt: 'Renaissance Technologies Medallion Fund strategy overview'</t>
+          <t>Lecture; Simulation Exercise (virtual order book); Case Excerpt: 'Renaissance Technologies Medallion Fund'</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="C30" s="83" t="inlineStr">
         <is>
-          <t>Backtesting Methodology &amp; Risk Metrics: Walk-forward backtesting vs. in-sample/out-of-sample testing; overfitting and data snooping bias; performance metrics: Sharpe ratio, Sortino ratio, Maximum Drawdown, Calmar ratio; transaction cost modelling; Case Discussion: 'Knight Capital Group $440M algorithmic trading failure – August 2012'.</t>
+          <t>[Hour 2] Backtesting Methodology &amp; Case Study: Walk-forward vs. in-sample/out-of-sample testing; overfitting and data snooping bias; Sharpe ratio, Sortino ratio, Maximum Drawdown; Case Discussion: 'Knight Capital Group $440M algorithmic trading failure – August 2012'.</t>
         </is>
       </c>
       <c r="D30" s="84" t="inlineStr">
         <is>
-          <t>Case Discussion; Quantitative Exercise (compute Sharpe ratio and Max Drawdown from return series); Peer Analysis presentation</t>
+          <t>Case Discussion; Quantitative Exercise (compute Sharpe ratio and Max Drawdown); Peer Analysis</t>
         </is>
       </c>
     </row>
@@ -1722,12 +1722,12 @@
       </c>
       <c r="C31" s="28" t="inlineStr">
         <is>
-          <t>AI-Enhanced Execution Strategies Lab: Reinforcement learning concepts (DQN, PPO) applied to trading; NLP-based signal generation from financial news; Lab: Build an AI trading bot using Backtrader + Python implementing a momentum strategy on NSE-listed stocks with full backtested results, Sharpe ratio, and drawdown report.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build an AI trading bot using Backtrader + Python (VS Code) — momentum strategy on NSE stocks with 2 years of data; generate full backtested performance report (Sharpe, CAGR, Max Drawdown); NLP-based signal from financial news.</t>
         </is>
       </c>
       <c r="D31" s="29" t="inlineStr">
         <is>
-          <t>Sandbox Lab (Backtrader + yfinance + Python); Peer Performance Review (compare strategy results across groups)</t>
+          <t>In-Class Python Lab (VS Code + Backtrader + yfinance); Peer Performance Review</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Module 5: Risk Modelling – PD Models &amp; Monte Carlo VaR</t>
+          <t>Session 5 (3 hrs) | Module 5: Risk Modelling – PD Models &amp; Monte Carlo VaR</t>
         </is>
       </c>
       <c r="B33" s="17" t="n">
@@ -1756,12 +1756,12 @@
       </c>
       <c r="C33" s="83" t="inlineStr">
         <is>
-          <t>Credit Risk Fundamentals &amp; PD Modelling: Credit risk components – Probability of Default (PD), Loss Given Default (LGD), Exposure at Default (EAD); Basel II Internal Ratings-Based (IRB) approach; ML-based PD models using logistic regression, decision trees, and XGBoost; feature engineering from financial ratios; handling class imbalance with SMOTE.</t>
+          <t>[Hour 1] Credit Risk &amp; PD Models: PD, LGD, EAD components; Basel II IRB approach; ML-based PD using logistic regression, decision trees, XGBoost; feature engineering from financial ratios; validation — Gini, KS statistic, AUC-ROC; SHAP for explainability; Case: 'Fintech lender PD model failure and NBFC regulatory action'.</t>
         </is>
       </c>
       <c r="D33" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Python Demo (scikit-learn credit model); Group Exercise: identify 10 key PD features for an Indian SME borrower</t>
+          <t>Lecture; Python Demo (scikit-learn); Case Discussion; SHAP Visualization Demo in Python (VS Code)</t>
         </is>
       </c>
     </row>
@@ -1772,12 +1772,12 @@
       </c>
       <c r="C34" s="83" t="inlineStr">
         <is>
-          <t>Credit Scorecard Validation &amp; Explainability: Scorecard development and points scaling; model validation metrics – Gini coefficient, KS statistic, AUC-ROC curve, Population Stability Index (PSI); SHAP values for model explainability and regulatory compliance; Case: 'Fintech lender PD model failure and NBFC regulatory action – lessons from Lending Fintech India 2023'.</t>
+          <t>[Hour 2] Monte Carlo VaR: Historical simulation vs. parametric vs. Monte Carlo compared; 10,000-path simulation for multi-asset portfolio; CVaR/Expected Shortfall; risk decomposition by asset; Basel III VaR thresholds (95%, 99%); Assignment introduced this session.</t>
         </is>
       </c>
       <c r="D34" s="84" t="inlineStr">
         <is>
-          <t>Case Discussion; Lab Exercise (SHAP visualizations in Python); Peer Review of model validation output</t>
+          <t>Lecture; Industry Simulation (multi-asset portfolio VaR); Risk Interpretation Workshop</t>
         </is>
       </c>
     </row>
@@ -1788,19 +1788,19 @@
       </c>
       <c r="C35" s="83" t="inlineStr">
         <is>
-          <t>Monte Carlo VaR Lab: Market risk measurement – historical simulation, parametric (variance-covariance), and Monte Carlo approaches compared; 10,000-path Monte Carlo simulation for a 5-stock NSE equity portfolio; Conditional VaR (CVaR) / Expected Shortfall (ES); risk decomposition by asset contribution; Lab: Generate a formatted VaR report with AI-written risk commentary using Claude API.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a Monte Carlo VaR engine in Python (VS Code + NumPy) for a 5-stock NSE portfolio; run 10,000 simulation paths; compute 95% and 99% VaR and CVaR; generate AI-written risk commentary using Claude API; output: formatted PDF report.</t>
         </is>
       </c>
       <c r="D35" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (NumPy + Monte Carlo simulation + Claude API); Risk Interpretation Workshop; results compared against 99% Basel III VaR threshold</t>
+          <t>In-Class Python Lab (VS Code + NumPy + Claude API + reportlab); Peer Report Review</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>Module 6: RegTech &amp; Automated Basel III/IV Compliance</t>
+          <t>Session 6 (3 hrs) | Module 6: RegTech &amp; Automated Basel III/IV Compliance</t>
         </is>
       </c>
       <c r="B36" s="21" t="n">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="C36" s="83" t="inlineStr">
         <is>
-          <t>Regulatory Framework – Basel III/IV: Capital adequacy ratios: CET1, Tier 1, Total Capital; Liquidity Coverage Ratio (LCR) and Net Stable Funding Ratio (NSFR); leverage ratio requirement; Basel IV Fundamental Review of the Trading Book (FRTB); RBI master circular on capital adequacy for Indian banks; AI applications in continuous compliance monitoring.</t>
+          <t>[Hour 1] Regulatory Framework – Basel III/IV: CET1, Tier 1, Total Capital adequacy ratios; LCR and NSFR; leverage ratio; Basel IV FRTB overview; RBI master circular for Indian banks; AI applications in continuous compliance monitoring; AxiomSL and OneSumX platforms.</t>
         </is>
       </c>
       <c r="D36" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Regulatory Simulation (AxiomSL-style capital calculation template); Guest Segment: RegTech industry overview video</t>
+          <t>Lecture; Regulatory Simulation (AxiomSL-style capital calculation template); Guest Video Segment</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="C37" s="83" t="inlineStr">
         <is>
-          <t>AML, KYC &amp; Regulatory Reporting Automation: Anti-Money Laundering (AML) transaction monitoring using ML; KYC automation using NLP (Aadhaar/PAN document processing); Suspicious Activity Report (SAR) auto-generation; FATF Recommendations 10 and 20; RBI guidelines on AI in banking; Case: 'HDFC Bank ₹1,000 crore RBI penalty – KYC compliance failure analysis'.</t>
+          <t>[Hour 2] AML, KYC &amp; Reporting Automation: AML transaction monitoring using ML; KYC document automation using NLP (Aadhaar/PAN OCR); SAR auto-generation; FATF Recommendations; Case: 'HDFC Bank Rs.1,000 crore RBI penalty – KYC compliance failure analysis'.</t>
         </is>
       </c>
       <c r="D37" s="84" t="inlineStr">
@@ -1840,12 +1840,12 @@
       </c>
       <c r="C38" s="83" t="inlineStr">
         <is>
-          <t>Pillar 3 Disclosure Automation Lab: Structure of Basel III Pillar 3 disclosure reports; extracting capital, risk, and liquidity data from structured bank financials; document generation pipeline architecture; Lab: Auto-generate a complete Basel III Pillar 3 disclosure document from bank data using Claude API and Python (output: formatted Word/PDF document).</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Auto-generate a Basel III Pillar 3 disclosure document from structured bank data using Claude API and Python (VS Code + python-docx); extract capital, risk, and liquidity metrics; produce formatted Word document matching RBI Pillar 3 template; peer review.</t>
         </is>
       </c>
       <c r="D38" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (Claude API + Python + python-docx); Peer Review of generated disclosures against RBI Pillar 3 template</t>
+          <t>In-Class Python Lab (VS Code + Claude API + python-docx); Peer Review of generated disclosures</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Module 7: Enterprise AI Governance, Security &amp; Cost Management</t>
+          <t>Session 7 (3 hrs) | Module 7: Enterprise AI Governance, Security &amp; Cost Management</t>
         </is>
       </c>
       <c r="B41" s="17" t="n">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="C41" s="83" t="inlineStr">
         <is>
-          <t>Model Risk Management &amp; AI Governance: Federal Reserve SR 11-7 model risk management framework; model documentation, independent validation, ongoing monitoring; AI explainability: SHAP vs LIME comparison; algorithmic bias and fairness in credit, insurance, and hiring; SEBI and RBI AI governance guidance; Case: 'Goldman Sachs Apple Card gender bias – CFPB investigation 2019'.</t>
+          <t>[Hour 1] AI Governance &amp; Model Risk Management: Federal Reserve SR 11-7 framework; model documentation, independent validation; SHAP and LIME for explainability; algorithmic bias and fairness; Case: 'Goldman Sachs Apple Card gender bias – CFPB investigation 2019'.</t>
         </is>
       </c>
       <c r="D41" s="84" t="inlineStr">
         <is>
-          <t>Case Discussion; AI Governance Framework Workshop; SHAP Visualization Demo in Python</t>
+          <t>Case Discussion; Governance Blueprint Workshop; SHAP Visualization Demo in Python (VS Code)</t>
         </is>
       </c>
     </row>
@@ -1894,12 +1894,12 @@
       </c>
       <c r="C42" s="83" t="inlineStr">
         <is>
-          <t>AI Regulation, Ethics &amp; Security: EU AI Act classification for financial services – prohibited, high-risk, limited-risk systems; India DPDP Act 2023 and financial data handling; Prompt injection attacks: direct and indirect; jailbreaking and model manipulation risks; OWASP LLM Top 10; data poisoning, model extraction, and model inversion attacks in finance.</t>
+          <t>[Hour 2 – Case Study] AI Security, Ethics &amp; Cost: EU AI Act classification for financial services; India DPDP Act 2023; prompt injection attacks (direct and indirect); OWASP LLM Top 10; TCO modelling (API costs, compute, integration, maintenance); Case Study: 'EisnerAmper GCC Pune – Automating Audit Analytics with Generative AI' (conducted in-class).</t>
         </is>
       </c>
       <c r="D42" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Red-Team Security Exercise (live prompt injection lab); Regulatory Comparison Table Workshop (EU AI Act vs SEBI vs RBI)</t>
+          <t>Case Study Discussion (in-class, 45 min); Red-Team Security Exercise (prompt injection); TCO Spreadsheet Modelling</t>
         </is>
       </c>
     </row>
@@ -1910,19 +1910,19 @@
       </c>
       <c r="C43" s="83" t="inlineStr">
         <is>
-          <t>AI Governance Blueprint &amp; TCO Lab: Total Cost of Ownership (TCO) modelling: API usage costs, compute, storage, integration, human oversight, and maintenance; cost optimization strategies – prompt caching, context compression, model routing, batching; Lab: Design a comprehensive AI Governance Blueprint for a bank deploying an LLM-based credit decision system, covering model risk, data privacy, bias testing, and incident response.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Design an AI Governance Blueprint for a bank deploying an LLM-based credit decision system — covering model risk, data privacy, bias testing, and incident response; build TCO model in Excel; group presentations (5 min each).</t>
         </is>
       </c>
       <c r="D43" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (TCO Excel Model + Claude API + Governance Blueprint document); Peer Presentation (5-min per group)</t>
+          <t>In-Class Workshop (Excel TCO + Claude API + Word Blueprint); Peer Presentations</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>Module 8: Fund Administration – NAV &amp; Transfer Agency Automation</t>
+          <t>Session 8 (3 hrs) | Module 8: Fund Administration – NAV &amp; Transfer Agency Automation</t>
         </is>
       </c>
       <c r="B44" s="21" t="n">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="C44" s="83" t="inlineStr">
         <is>
-          <t>Fund Administration Lifecycle: Fund types (mutual funds, hedge funds, PE/VC, AIFs, REITs); trade capture and confirmation workflow; portfolio valuation methods (mark-to-market, mark-to-model, IFRS 9); corporate actions processing; NAV calculation steps; investor reporting; AI applications in fund accounting at Opus Fund Services, HC Global, SS&amp;C GlobeOp, and Apex Group.</t>
+          <t>[Hour 1] Fund Administration Lifecycle: Fund types (mutual funds, hedge funds, PE/VC, AIFs); trade capture, portfolio valuation (mark-to-market, IFRS 9), corporate actions, NAV calculation; investor reporting; AI applications at Opus Fund Services, HC Global, SS&amp;C GlobeOp, Apex Group; Case: 'Opus Fund Services AI-powered fund automation GCC Pune'.</t>
         </is>
       </c>
       <c r="D44" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Industry Case: 'Opus Fund Services – AI-powered fund automation GCC Pune'; Role-Mapping Exercise (identify AI insertion points in fund lifecycle)</t>
+          <t>Lecture; Industry Case Discussion; Role-Mapping Exercise (identify AI insertion points in fund lifecycle)</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1946,12 @@
       </c>
       <c r="C45" s="83" t="inlineStr">
         <is>
-          <t>Transfer Agency &amp; KYC Operations: Transfer agency workflow – investor onboarding, subscription and redemption processing, dividend distribution, statement generation; AML/KYC for fund investors using NLP – Aadhaar-based e-KYC, PAN verification, document OCR; SEBI mutual fund KYC regulations 2023; KFINTECH and CAMS platforms; STP (Straight-Through Processing) and error reconciliation.</t>
+          <t>[Hour 2] Transfer Agency &amp; KYC Automation: Investor onboarding (AML/KYC), subscription/redemption processing, dividend distribution; Aadhaar-based e-KYC and PAN verification using NLP; SEBI mutual fund KYC regulations 2023; KFINTECH and CAMS platforms; STP and error reconciliation.</t>
         </is>
       </c>
       <c r="D45" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Role-Play Exercise (investor onboarding simulation with mock KYC documents); KYC NLP Demo (document classification)</t>
+          <t>Lecture; Role-Play Exercise (investor onboarding simulation with mock KYC documents); KYC NLP Demo</t>
         </is>
       </c>
     </row>
@@ -1962,19 +1962,19 @@
       </c>
       <c r="C46" s="83" t="inlineStr">
         <is>
-          <t>NAV Automation Lab: Lab – Build a Python-based daily NAV calculation engine for a hypothetical equity mutual fund with 10 NSE-listed holdings; auto-generate an AI-written daily fund manager commentary and NAV report using Claude API; include reconciliation check automation; output: formatted Excel/PDF report matching SEBI disclosure format.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a Python-based NAV calculation engine (VS Code) for a 10-holding equity mutual fund; auto-generate a daily fund manager commentary and NAV report using Claude API; implement reconciliation check; output: formatted Excel/PDF report matching SEBI disclosure format.</t>
         </is>
       </c>
       <c r="D46" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (Python + Claude API + openpyxl/reportlab); Peer Review (evaluate NAV accuracy and commentary quality)</t>
+          <t>In-Class Python Lab (VS Code + Claude API + openpyxl + reportlab); Peer Review (NAV accuracy and commentary quality)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1" thickBot="1">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Module 9: Market Commentary &amp; Valuation Dashboards</t>
+          <t>Session 9 (3 hrs) | Module 9: Market Commentary &amp; Valuation Dashboards</t>
         </is>
       </c>
       <c r="B47" s="17" t="n">
@@ -1982,12 +1982,12 @@
       </c>
       <c r="C47" s="83" t="inlineStr">
         <is>
-          <t>Financial NLP – Sentiment Analysis &amp; Market Commentary: FinBERT for financial sentiment analysis; earnings call transcript mining and key phrase extraction; Bloomberg NLP applications in market intelligence; news-based event-driven trading signals; NLP pipeline: NSE announcement collection → preprocessing → FinBERT sentiment scoring → AI-generated equity research commentary.</t>
+          <t>[Hour 1] Financial NLP &amp; Sentiment Analysis: FinBERT for financial sentiment; earnings call transcript mining; Bloomberg NLP use-cases; news-based event-driven signals; NLP pipeline — NSE announcement collection → preprocessing → FinBERT scoring → AI-generated equity research commentary; Case: 'Bloomberg Intelligence AI-generated earnings summaries'.</t>
         </is>
       </c>
       <c r="D47" s="84" t="inlineStr">
         <is>
-          <t>Lecture; Live Demo (FinBERT on NSE earnings transcript); Case: 'Bloomberg Intelligence – AI-generated earnings summaries'</t>
+          <t>Lecture; Live Demo (FinBERT on NSE earnings transcript); Case Discussion</t>
         </is>
       </c>
     </row>
@@ -2012,12 +2012,12 @@
       </c>
       <c r="C49" s="32" t="inlineStr">
         <is>
-          <t>Valuation Modelling with AI Assistance: DCF (Discounted Cash Flow) model automation using Claude API – revenue projection, WACC calculation, terminal value; Comparable Company Analysis (CCA) automation: extract and compare EV/EBITDA, P/E, P/BV multiples; ESG data integration in equity valuation; Damodaran valuation database application; valuation exercise on a real NSE-listed company.</t>
+          <t>[Hour 2] Valuation Modelling with AI: DCF model automation using Claude API — revenue projection, WACC, terminal value; CCA automation — extract and compare EV/EBITDA, P/E, P/BV multiples; ESG data integration; Damodaran valuation database; live valuation exercise on NSE-listed company.</t>
         </is>
       </c>
       <c r="D49" s="33" t="inlineStr">
         <is>
-          <t>Modelling Lab (Python-based DCF + Claude API for narrative); Case: Valuation of TCS / Infosys using CCA and DCF</t>
+          <t>Modelling Lab (Python-based DCF + Claude API in VS Code); Live Company Valuation Exercise</t>
         </is>
       </c>
     </row>
@@ -2028,19 +2028,19 @@
       </c>
       <c r="C50" s="83" t="inlineStr">
         <is>
-          <t>Streamlit Market Intelligence Dashboard Lab: Streamlit framework for financial dashboards; Plotly for interactive charts (candlestick, heatmap, portfolio performance chart); real-time market data integration (NSE API, Yahoo Finance); Lab: Build a complete Streamlit market intelligence dashboard with a stock screener, portfolio analytics panel, and FinBERT sentiment feed.</t>
+          <t>[Hour 3 – Lab] In-Class Lab: Build a Streamlit market intelligence dashboard (VS Code) with — stock screener, candlestick charts (Plotly), portfolio analytics panel, and FinBERT sentiment feed from NSE news; integrate real-time data (yfinance); peer review for usability and data accuracy.</t>
         </is>
       </c>
       <c r="D50" s="84" t="inlineStr">
         <is>
-          <t>Sandbox Lab (Streamlit + Plotly + yfinance + FinBERT); Live Demo; Peer Review (usability and data accuracy)</t>
+          <t>In-Class Python Lab (VS Code + Streamlit + Plotly + yfinance + FinBERT); Live Demo; Peer Review</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Module 10: GCC Capstone – Integrated Financial AI System</t>
+          <t>Session 10 (3 hrs) | Module 10: GCC Capstone – Integrated Financial AI System</t>
         </is>
       </c>
       <c r="B51" s="17" t="n">
@@ -2048,12 +2048,12 @@
       </c>
       <c r="C51" s="83" t="inlineStr">
         <is>
-          <t>Capstone Integration &amp; Architecture: Combine all module deliverables (RAG prospectus bot, Monte Carlo VaR engine, NAV automation, Basel III disclosure generator, Streamlit dashboard) into a unified Integrated Financial AI System; system architecture documentation; integration testing; GitHub repository setup; capstone rubric walkthrough.</t>
+          <t>[Hour 1] Capstone Integration: Combine all module deliverables (RAG prospectus bot, Monte Carlo VaR engine, Basel III disclosure generator, NAV automation, Streamlit dashboard) into a unified Integrated Financial AI System; system architecture documentation; integration testing; GitHub portfolio setup; capstone rubric walkthrough.</t>
         </is>
       </c>
       <c r="D51" s="84" t="inlineStr">
         <is>
-          <t>Workshop (Instructor-led integration session + Peer Review rounds); Integration Lab; GitHub portfolio setup guidance</t>
+          <t>Workshop (Instructor-led integration session + Peer Review rounds); Integration Lab; GitHub Setup</t>
         </is>
       </c>
     </row>
@@ -2064,12 +2064,12 @@
       </c>
       <c r="C52" s="83" t="inlineStr">
         <is>
-          <t>Pitch Deck Design &amp; Mock Rehearsal: Pitch deck structure for GCC hiring panels: Problem → Solution Architecture → Live Demo → Business Impact → Team; AI-assisted resume and cover letter tailoring for GCC finance + AI roles; common technical interview questions (Python, finance, AI governance); structured peer rehearsal with feedback rubric.</t>
+          <t>[Hour 2] Pitch Deck Design &amp; Mock Rehearsal: Pitch deck structure for GCC hiring panels — Problem → Solution Architecture → Live Demo → Business Impact → Team; AI-assisted resume and cover letter tailoring; technical interview preparation (Python, finance, AI governance); structured peer rehearsal with GCC hiring rubric feedback.</t>
         </is>
       </c>
       <c r="D52" s="84" t="inlineStr">
         <is>
-          <t>Group Rehearsal; Structured Peer Feedback (using GCC hiring rubric); Instructor Coaching round</t>
+          <t>Group Rehearsal; Structured Peer Feedback (GCC hiring rubric); Instructor Coaching Round</t>
         </is>
       </c>
     </row>
@@ -2080,12 +2080,12 @@
       </c>
       <c r="C53" s="83" t="inlineStr">
         <is>
-          <t>GCC Capstone Presentation: Live 15-minute project presentation to mock GCC hiring panel (EisnerAmper / Opus Fund Services scenario); 10-minute Q&amp;A with panel (faculty in role of GCC managers); placement readiness scoring on: technical depth, communication, portfolio quality, and role alignment; individual feedback; course debrief – industry outlook and next steps.</t>
+          <t>[Hour 3 – Capstone] GCC Capstone Presentation: Live 15-minute project presentation to mock GCC hiring panel (EisnerAmper/Opus Fund Services scenario); 10-minute Q&amp;A; placement readiness scoring on technical depth, communication, portfolio quality, and role alignment; individual feedback; course debrief.</t>
         </is>
       </c>
       <c r="D53" s="84" t="inlineStr">
         <is>
-          <t>Mock Hiring Panel (faculty role-play as GCC panel); Peer Evaluation Rubric; Course Debrief Discussion; individual feedback forms</t>
+          <t>Mock Hiring Panel (faculty as GCC panel); Peer Evaluation Rubric; Course Debrief Discussion</t>
         </is>
       </c>
     </row>

</xml_diff>